<commit_message>
last change before switching to standards
</commit_message>
<xml_diff>
--- a/assets/excel/template_charts.xlsx
+++ b/assets/excel/template_charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grouperenault-my.sharepoint.com/personal/lola_gauducheau_renault_com/Documents/Documents/suivi_chrono/assets/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="127" documentId="8_{F52C1A9A-D12F-48B6-B6D3-92EE9EABD670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D723771C-6B3E-4588-AD5B-912AFB640E3C}"/>
+  <xr:revisionPtr revIDLastSave="142" documentId="8_{F52C1A9A-D12F-48B6-B6D3-92EE9EABD670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7B8F248-497F-4ECF-B556-2A9B8D6B378E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw" sheetId="4" r:id="rId1"/>
@@ -32,7 +32,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId8"/>
+    <pivotCache cacheId="0" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -210,7 +210,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="hh:mm:ss.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="hh:mm:ss.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
@@ -222,12 +231,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="hh:mm:ss.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="hh:mm:ss.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="hh:mm:ss.00"/>
@@ -3249,7 +3252,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C5BE52AF-34F3-44DA-9999-46BD60685536}" name="Tableau croisé dynamique1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C5BE52AF-34F3-44DA-9999-46BD60685536}" name="Tableau croisé dynamique1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" showAll="0">
@@ -3307,12 +3310,14 @@
     <tableColumn id="1" xr3:uid="{36F4E5C7-C9AD-477E-836A-7EC9C1E5F5C2}" name="Tâche"/>
     <tableColumn id="2" xr3:uid="{5D82B2A6-E46B-4DD9-8367-94DE63E019F6}" name="Début (valeur Excel date+heure"/>
     <tableColumn id="3" xr3:uid="{AD77BDF4-D552-422F-A5DB-75BA1A879FFA}" name="Fin (valeur Excel date+heure)"/>
-    <tableColumn id="4" xr3:uid="{BA31084A-5920-41D7-BF2E-D0B8836FB771}" name="Durée (peut être texte ou valeur)"/>
+    <tableColumn id="4" xr3:uid="{BA31084A-5920-41D7-BF2E-D0B8836FB771}" name="Durée (peut être texte ou valeur)" dataDxfId="0">
+      <calculatedColumnFormula>(C2-B2)</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="5" xr3:uid="{CE0CD001-58CA-47EE-A2FD-9DDD9441B668}" name="VA/NVA"/>
-    <tableColumn id="6" xr3:uid="{B71CADA4-38F2-4FEE-8102-35158BD92733}" name="Durée (jours)" dataDxfId="9">
+    <tableColumn id="6" xr3:uid="{B71CADA4-38F2-4FEE-8102-35158BD92733}" name="Durée (jours)" dataDxfId="11">
       <calculatedColumnFormula>IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{84FFCF15-EE45-4484-9503-C9F32AFAAC6C}" name="Durée (ms)" dataDxfId="8">
+    <tableColumn id="7" xr3:uid="{84FFCF15-EE45-4484-9503-C9F32AFAAC6C}" name="Durée (ms)" dataDxfId="10">
       <calculatedColumnFormula>IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{085153DF-BC56-4F3C-88F5-056E13E55BAF}" name="Durée (affichage)"/>
@@ -3325,28 +3330,28 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F13784D2-8AE6-4C5A-8E4D-CA1B904EFFC5}" name="Tableau5" displayName="Tableau5" ref="A1:H200" totalsRowShown="0">
   <autoFilter ref="A1:H200" xr:uid="{F13784D2-8AE6-4C5A-8E4D-CA1B904EFFC5}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1E4A0DCE-4F01-4D90-9041-0CA1A039F98D}" name="Tâche" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{1E4A0DCE-4F01-4D90-9041-0CA1A039F98D}" name="Tâche" dataDxfId="9">
       <calculatedColumnFormula array="1">_xlfn.UNIQUE(TableRaw[Tâche])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A2C3D671-E00C-436D-8118-37C1ABBFBAF4}" name="Occurrences" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{A2C3D671-E00C-436D-8118-37C1ABBFBAF4}" name="Occurrences" dataDxfId="8">
       <calculatedColumnFormula>COUNTIF(TableRaw[Tâche], A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EF0E5F4F-97C7-4792-A47E-9DEA80F91F82}" name="Temps total" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{EF0E5F4F-97C7-4792-A47E-9DEA80F91F82}" name="Temps total" dataDxfId="7">
       <calculatedColumnFormula>SUMIF(TableRaw[Tâche], A2, TableRaw[Durée (jours)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7CEEF28F-92BD-4603-B501-364D5052FDCD}" name="Temps moyen" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{7CEEF28F-92BD-4603-B501-364D5052FDCD}" name="Temps moyen" dataDxfId="6">
       <calculatedColumnFormula>IF(B2=0,"",C2/B2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DC432A1F-B490-4482-8F6E-D01688363439}" name="Temps min" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{DC432A1F-B490-4482-8F6E-D01688363439}" name="Temps min" dataDxfId="5">
       <calculatedColumnFormula array="1">IFERROR(MIN(IF(TableRaw[Tâche]=A2,TableRaw[Durée (jours)])),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{2CA7E18F-F0B1-4824-A5F3-712E3F28B55F}" name="Temps max" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{2CA7E18F-F0B1-4824-A5F3-712E3F28B55F}" name="Temps max" dataDxfId="4">
       <calculatedColumnFormula array="1">IFERROR(LARGE(IF(TableRaw[Tâche]=A2,TableRaw[Durée (jours)]),1),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{B45871F3-F27D-44F3-95CE-531A6B67BE97}" name="% du temps total" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{B45871F3-F27D-44F3-95CE-531A6B67BE97}" name="% du temps total" dataDxfId="3">
       <calculatedColumnFormula>IF($H$2=0,"",C2 / $H$2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{41C1C735-FA47-40A8-A10A-8ED90EE487B6}" name="Total session (jours)" dataDxfId="6">
+    <tableColumn id="8" xr3:uid="{41C1C735-FA47-40A8-A10A-8ED90EE487B6}" name="Total session (jours)" dataDxfId="2">
       <calculatedColumnFormula>SUM(TableRaw[Durée (jours)])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3361,7 +3366,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Tâche"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Début"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Fin"/>
-    <tableColumn id="4" xr3:uid="{BED66CE7-4585-4048-A3FF-D5E4025BDA4B}" name="Durée" dataDxfId="10">
+    <tableColumn id="4" xr3:uid="{BED66CE7-4585-4048-A3FF-D5E4025BDA4B}" name="Durée" dataDxfId="1">
       <calculatedColumnFormula>IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{6671B2A2-1F41-4601-BCBB-7B19829987AF}" name="VA/NVA"/>
@@ -3660,7 +3665,7 @@
   <cols>
     <col min="2" max="2" width="29.08984375" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="30.54296875" customWidth="1"/>
+    <col min="4" max="4" width="30.54296875" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.7265625" customWidth="1"/>
     <col min="7" max="7" width="13.36328125" customWidth="1"/>
     <col min="8" max="8" width="17.453125" customWidth="1"/>
@@ -3676,7 +3681,7 @@
       <c r="C1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E1" t="s">
@@ -3693,1992 +3698,2788 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D2" s="1">
+        <f t="shared" ref="D2:D33" si="0">(C2-B2)</f>
+        <v>0</v>
+      </c>
       <c r="F2" t="str">
-        <f t="shared" ref="F2:F33" si="0">IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</f>
+        <f t="shared" ref="F2:F33" si="1">IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</f>
         <v/>
       </c>
       <c r="G2" s="1" t="str">
-        <f t="shared" ref="G2:G65" si="1">IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</f>
+        <f t="shared" ref="G2:G65" si="2">IF(AND(B2&lt;&gt;"",C2&lt;&gt;""),C2-B2,"")</f>
         <v/>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D3" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="F3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G3" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D4" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G3" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F4" t="str">
+      <c r="G4" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D5" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G4" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F5" t="str">
+      <c r="G5" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D6" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G5" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F6" t="str">
+      <c r="G6" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D7" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G6" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F7" t="str">
+      <c r="G7" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D8" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G7" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F8" t="str">
+      <c r="G8" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D9" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G8" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F9" t="str">
+      <c r="G9" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D10" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G9" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F10" t="str">
+      <c r="G10" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D11" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G10" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F11" t="str">
+      <c r="G11" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D12" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G11" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F12" t="str">
+      <c r="G12" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D13" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G12" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F13" t="str">
+      <c r="G13" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D14" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G13" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F14" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F14" t="str">
+      <c r="G14" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D15" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G14" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F15" t="str">
+      <c r="G15" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D16" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G15" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F16" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F16" t="str">
+      <c r="G16" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D17" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G16" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="17" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F17" t="str">
+      <c r="G17" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D18" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G17" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="18" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F18" t="str">
+      <c r="G18" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D19" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G18" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F19" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="19" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F19" t="str">
+      <c r="G19" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D20" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G19" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="20" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F20" t="str">
+      <c r="G20" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D21" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G20" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="21" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F21" t="str">
+      <c r="G21" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D22" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G21" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F22" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="22" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F22" t="str">
+      <c r="G22" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D23" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G22" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="23" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F23" t="str">
+      <c r="G23" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D24" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G23" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F24" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="24" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F24" t="str">
+      <c r="G24" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D25" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G24" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F25" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="25" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F25" t="str">
+      <c r="G25" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D26" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G25" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F26" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="26" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F26" t="str">
+      <c r="G26" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D27" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G26" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="27" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F27" t="str">
+      <c r="G27" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D28" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G27" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="28" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F28" t="str">
+      <c r="G28" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D29" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G28" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F29" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="29" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F29" t="str">
+      <c r="G29" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D30" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G29" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="30" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F30" t="str">
+      <c r="G30" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D31" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G30" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="31" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F31" t="str">
+      <c r="G31" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D32" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G31" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F32" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="32" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F32" t="str">
+      <c r="G32" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D33" s="1">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G32" s="1" t="str">
+        <v>0</v>
+      </c>
+      <c r="F33" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="33" spans="6:7" x14ac:dyDescent="0.35">
-      <c r="F33" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="G33" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D34" s="1">
+        <f t="shared" ref="D34:D65" si="3">(C34-B34)</f>
+        <v>0</v>
+      </c>
       <c r="F34" t="str">
-        <f t="shared" ref="F34:F65" si="2">IF(AND(B34&lt;&gt;"",C34&lt;&gt;""),C34-B34,"")</f>
+        <f t="shared" ref="F34:F65" si="4">IF(AND(B34&lt;&gt;"",C34&lt;&gt;""),C34-B34,"")</f>
         <v/>
       </c>
       <c r="G34" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D35" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F35" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G35" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G35" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D36" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F36" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G36" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G36" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D37" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F37" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G37" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G37" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D38" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F38" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G38" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G38" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="39" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D39" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F39" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G39" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G39" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D40" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F40" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G40" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G40" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="41" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D41" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F41" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G41" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G41" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="42" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D42" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F42" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G42" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G42" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="43" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D43" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F43" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G43" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G43" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D44" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F44" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G44" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G44" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="45" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D45" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F45" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G45" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G45" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="46" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D46" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F46" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G46" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G46" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="47" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D47" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F47" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G47" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G47" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="48" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D48" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F48" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G48" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G48" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="49" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D49" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F49" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G49" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G49" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="50" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D50" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F50" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G50" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G50" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="51" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D51" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F51" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G51" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G51" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="52" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D52" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F52" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G52" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G52" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="53" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D53" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F53" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G53" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G53" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="54" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D54" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F54" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G54" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G54" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="55" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D55" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F55" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G55" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G55" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="56" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D56" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F56" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G56" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G56" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="57" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D57" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F57" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G57" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G57" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="58" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D58" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F58" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G58" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G58" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="59" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D59" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F59" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G59" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G59" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="60" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D60" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F60" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G60" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G60" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="61" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D61" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F61" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G61" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G61" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="62" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D62" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F62" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G62" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G62" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="63" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D63" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F63" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G63" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G63" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="64" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D64" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F64" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G64" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G64" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="65" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D65" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
       <c r="F65" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G65" s="1" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G65" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="6:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="66" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D66" s="1">
+        <f t="shared" ref="D66:D97" si="5">(C66-B66)</f>
+        <v>0</v>
+      </c>
       <c r="F66" t="str">
-        <f t="shared" ref="F66:F97" si="3">IF(AND(B66&lt;&gt;"",C66&lt;&gt;""),C66-B66,"")</f>
+        <f t="shared" ref="F66:F97" si="6">IF(AND(B66&lt;&gt;"",C66&lt;&gt;""),C66-B66,"")</f>
         <v/>
       </c>
       <c r="G66" s="1" t="str">
-        <f t="shared" ref="G66:G129" si="4">IF(AND(B66&lt;&gt;"",C66&lt;&gt;""),C66-B66,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" ref="G66:G129" si="7">IF(AND(B66&lt;&gt;"",C66&lt;&gt;""),C66-B66,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D67" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F67" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G67" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D68" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F68" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G68" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D69" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F69" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G69" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D70" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F70" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G70" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D71" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F71" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G71" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D72" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F72" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G72" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D73" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F73" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G73" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D74" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F74" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G74" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D75" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F75" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G75" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D76" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F76" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G76" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D77" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F77" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G77" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D78" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F78" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G78" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D79" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F79" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G79" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D80" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F80" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G80" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D81" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F81" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G81" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D82" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F82" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G82" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D83" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F83" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G83" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D84" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F84" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G84" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D85" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F85" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G85" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D86" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F86" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G86" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="87" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D87" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F87" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G87" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D88" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F88" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G88" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="89" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D89" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F89" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G89" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D90" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F90" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G90" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="91" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D91" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F91" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G91" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D92" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F92" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G92" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D93" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F93" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G93" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D94" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F94" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G94" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="95" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D95" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F95" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G95" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="96" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D96" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F96" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G96" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="97" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="97" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D97" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="F97" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="G97" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="98" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D98" s="1">
+        <f t="shared" ref="D98:D129" si="8">(C98-B98)</f>
+        <v>0</v>
+      </c>
       <c r="F98" t="str">
-        <f t="shared" ref="F98:F129" si="5">IF(AND(B98&lt;&gt;"",C98&lt;&gt;""),C98-B98,"")</f>
+        <f t="shared" ref="F98:F129" si="9">IF(AND(B98&lt;&gt;"",C98&lt;&gt;""),C98-B98,"")</f>
         <v/>
       </c>
       <c r="G98" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="99" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="99" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D99" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F99" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G99" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="100" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="100" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D100" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F100" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G100" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="101" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D101" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F101" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G101" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="102" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="102" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D102" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F102" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G102" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="103" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="103" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D103" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F103" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G103" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="104" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="104" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D104" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F104" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G104" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="105" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="105" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D105" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F105" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G105" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="106" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="106" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D106" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F106" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G106" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="107" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="107" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D107" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F107" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G107" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="108" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D108" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F108" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G108" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="109" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="109" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D109" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F109" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G109" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="110" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="110" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D110" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F110" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G110" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="111" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="111" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D111" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F111" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G111" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="112" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="112" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D112" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F112" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G112" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="113" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="113" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D113" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F113" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G113" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="114" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="114" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D114" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F114" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G114" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="115" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="115" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D115" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F115" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G115" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="116" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="116" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D116" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F116" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G116" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="117" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="117" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D117" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F117" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G117" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="118" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="118" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D118" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F118" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G118" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="119" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="119" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D119" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F119" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G119" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="120" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="120" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D120" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F120" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G120" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="121" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="121" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D121" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F121" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G121" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="122" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="122" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D122" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F122" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G122" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="123" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="123" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D123" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F123" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G123" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="124" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="124" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D124" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F124" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G124" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="125" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="125" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D125" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F125" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G125" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="126" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="126" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D126" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F126" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G126" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="127" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="127" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D127" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F127" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G127" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="128" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="128" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D128" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F128" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G128" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="129" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="129" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D129" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
       <c r="F129" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="G129" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="130" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="130" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D130" s="1">
+        <f t="shared" ref="D130:D161" si="10">(C130-B130)</f>
+        <v>0</v>
+      </c>
       <c r="F130" t="str">
-        <f t="shared" ref="F130:F161" si="6">IF(AND(B130&lt;&gt;"",C130&lt;&gt;""),C130-B130,"")</f>
+        <f t="shared" ref="F130:F161" si="11">IF(AND(B130&lt;&gt;"",C130&lt;&gt;""),C130-B130,"")</f>
         <v/>
       </c>
       <c r="G130" s="1" t="str">
-        <f t="shared" ref="G130:G193" si="7">IF(AND(B130&lt;&gt;"",C130&lt;&gt;""),C130-B130,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="131" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" ref="G130:G193" si="12">IF(AND(B130&lt;&gt;"",C130&lt;&gt;""),C130-B130,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D131" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F131" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G131" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="132" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="132" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D132" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F132" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G132" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="133" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="133" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D133" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F133" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G133" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="134" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="134" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D134" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F134" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G134" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="135" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="135" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D135" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F135" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G135" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="136" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="136" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D136" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F136" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G136" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="137" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="137" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D137" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F137" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G137" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="138" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="138" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D138" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F138" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G138" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="139" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="139" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D139" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F139" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G139" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="140" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="140" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D140" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F140" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G140" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="141" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="141" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D141" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F141" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G141" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="142" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="142" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D142" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F142" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G142" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="143" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="143" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D143" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F143" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G143" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="144" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="144" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D144" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F144" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G144" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="145" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="145" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D145" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F145" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G145" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="146" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="146" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D146" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F146" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G146" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="147" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="147" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D147" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F147" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G147" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="148" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="148" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D148" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F148" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G148" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="149" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="149" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D149" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F149" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G149" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="150" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="150" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D150" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F150" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G150" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="151" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="151" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D151" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F151" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G151" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="152" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="152" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D152" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F152" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G152" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="153" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="153" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D153" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F153" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G153" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="154" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="154" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D154" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F154" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G154" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="155" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="155" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D155" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F155" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G155" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="156" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="156" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D156" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F156" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G156" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="157" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="157" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D157" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F157" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G157" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="158" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="158" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D158" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F158" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G158" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="159" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="159" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D159" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F159" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G159" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="160" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="160" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D160" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F160" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G160" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="161" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="161" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D161" s="1">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="F161" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="G161" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="162" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="162" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D162" s="1">
+        <f t="shared" ref="D162:D193" si="13">(C162-B162)</f>
+        <v>0</v>
+      </c>
       <c r="F162" t="str">
-        <f t="shared" ref="F162:F193" si="8">IF(AND(B162&lt;&gt;"",C162&lt;&gt;""),C162-B162,"")</f>
+        <f t="shared" ref="F162:F193" si="14">IF(AND(B162&lt;&gt;"",C162&lt;&gt;""),C162-B162,"")</f>
         <v/>
       </c>
       <c r="G162" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="163" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="163" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D163" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F163" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G163" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="164" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="164" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D164" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F164" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G164" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="165" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="165" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D165" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F165" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G165" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="166" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="166" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D166" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F166" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G166" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="167" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="167" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D167" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F167" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G167" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="168" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="168" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D168" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F168" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G168" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="169" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="169" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D169" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F169" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G169" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="170" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="170" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D170" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F170" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G170" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="171" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="171" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D171" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F171" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G171" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="172" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="172" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D172" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F172" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G172" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="173" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="173" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D173" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F173" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G173" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="174" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="174" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D174" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F174" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G174" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="175" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="175" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D175" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F175" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G175" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="176" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="176" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D176" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F176" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G176" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="177" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="177" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D177" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F177" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G177" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="178" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="178" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D178" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F178" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G178" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="179" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="179" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D179" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F179" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G179" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="180" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="180" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D180" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F180" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G180" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="181" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="181" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D181" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F181" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G181" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="182" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="182" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D182" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F182" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G182" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="183" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="183" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D183" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F183" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G183" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="184" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="184" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D184" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F184" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G184" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="185" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="185" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D185" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F185" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G185" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="186" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="186" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D186" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F186" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G186" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="187" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="187" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D187" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F187" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G187" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="188" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="188" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D188" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F188" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G188" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="189" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="189" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D189" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F189" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G189" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="190" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="190" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D190" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F190" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G190" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="191" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="191" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D191" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F191" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G191" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="192" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="192" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D192" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F192" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G192" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="193" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="193" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D193" s="1">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
       <c r="F193" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="G193" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="194" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="194" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D194" s="1">
+        <f t="shared" ref="D194:D225" si="15">(C194-B194)</f>
+        <v>0</v>
+      </c>
       <c r="F194" t="str">
-        <f t="shared" ref="F194:F200" si="9">IF(AND(B194&lt;&gt;"",C194&lt;&gt;""),C194-B194,"")</f>
+        <f t="shared" ref="F194:F200" si="16">IF(AND(B194&lt;&gt;"",C194&lt;&gt;""),C194-B194,"")</f>
         <v/>
       </c>
       <c r="G194" s="1" t="str">
-        <f t="shared" ref="G194:G200" si="10">IF(AND(B194&lt;&gt;"",C194&lt;&gt;""),C194-B194,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="195" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" ref="G194:G200" si="17">IF(AND(B194&lt;&gt;"",C194&lt;&gt;""),C194-B194,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D195" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="F195" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="G195" s="1" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-    </row>
-    <row r="196" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="196" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D196" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="F196" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="G196" s="1" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-    </row>
-    <row r="197" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="197" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D197" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="F197" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="G197" s="1" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-    </row>
-    <row r="198" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="198" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D198" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="F198" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="G198" s="1" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-    </row>
-    <row r="199" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="199" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D199" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="F199" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="G199" s="1" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-    </row>
-    <row r="200" spans="6:7" x14ac:dyDescent="0.35">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+    </row>
+    <row r="200" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D200" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="F200" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="G200" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
     </row>

</xml_diff>